<commit_message>
Added iteration to spring and rectangle
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14644A70-6F27-4F12-B8FE-80EF415B7656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1275E27-73E6-403D-9BD4-03D7EEB982F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>Steel (1010 hot rolled)</t>
   </si>
   <si>
-    <t>Steel (4140 Q&amp;T @400</t>
-  </si>
-  <si>
     <t>Aluminum (1100 annealed)</t>
   </si>
   <si>
@@ -90,6 +87,9 @@
   </si>
   <si>
     <t>Kevlar (82 vol % in epoxy)</t>
+  </si>
+  <si>
+    <t>Steel (4140 Q&amp;T @400)</t>
   </si>
 </sst>
 </file>
@@ -474,16 +474,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -505,7 +505,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>30000000</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>10400000</v>
@@ -539,7 +539,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>10400000</v>
@@ -556,7 +556,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>16500000</v>
@@ -573,7 +573,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>16500000</v>
@@ -590,7 +590,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8">
         <v>18500000</v>
@@ -607,7 +607,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>24500000</v>
@@ -624,7 +624,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10">
         <v>200000</v>
@@ -641,7 +641,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>400000</v>
@@ -658,7 +658,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>200000</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>12000000</v>
@@ -692,7 +692,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14">
         <v>8100000</v>

</xml_diff>

<commit_message>
Added iteration to circle and rectangle. Also added PLA to materials sheet
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1275E27-73E6-403D-9BD4-03D7EEB982F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A911ED7-841D-436C-861E-2FF87BC15674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Material</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Steel (4140 Q&amp;T @400)</t>
+  </si>
+  <si>
+    <t>PLA</t>
   </si>
 </sst>
 </file>
@@ -462,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CDE8C3E-D2CD-4FEC-B8FA-734CEE576120}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
@@ -707,6 +710,23 @@
         <v>1640000000</v>
       </c>
     </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15">
+        <v>400000</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>8000</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added code to separate failure from success and added some materials to the database
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A911ED7-841D-436C-861E-2FF87BC15674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8523038A-B4A6-4FBD-9A16-05D72736148B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Material</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>PLA</t>
+  </si>
+  <si>
+    <t>Delrin</t>
+  </si>
+  <si>
+    <t>ABS</t>
   </si>
 </sst>
 </file>
@@ -465,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CDE8C3E-D2CD-4FEC-B8FA-734CEE576120}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
@@ -727,6 +733,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16">
+        <v>500000</v>
+      </c>
+      <c r="C16" s="1">
+        <v>3250000000</v>
+      </c>
+      <c r="D16" s="1">
+        <v>12000</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="1">
+        <v>325000</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>7000</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Stainless Steel to Database and updated geometry for wire
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8523038A-B4A6-4FBD-9A16-05D72736148B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E92ED6-0FFD-4300-B03E-58BDB467ECA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Material</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>ABS</t>
+  </si>
+  <si>
+    <t>304 Stainless Steel (Q&amp;T)</t>
   </si>
 </sst>
 </file>
@@ -471,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CDE8C3E-D2CD-4FEC-B8FA-734CEE576120}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
@@ -767,6 +770,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="1">
+        <v>28000000</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1">
+        <v>45000</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added another version of Stainless Steel
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E92ED6-0FFD-4300-B03E-58BDB467ECA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78938A3-8943-416B-9BA9-4B605EF170B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Material</t>
   </si>
@@ -101,7 +101,10 @@
     <t>ABS</t>
   </si>
   <si>
-    <t>304 Stainless Steel (Q&amp;T)</t>
+    <t>304 Stainless Steel CD</t>
+  </si>
+  <si>
+    <t>304 Stainless Steel Annealed</t>
   </si>
 </sst>
 </file>
@@ -474,10 +477,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CDE8C3E-D2CD-4FEC-B8FA-734CEE576120}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -787,6 +790,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="1">
+        <v>28000000</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>29700</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Galvanized Steel and return of alternating stress
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78938A3-8943-416B-9BA9-4B605EF170B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D76C94-FCC6-4518-AE59-C19DA35C5E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Material</t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t>304 Stainless Steel Annealed</t>
+  </si>
+  <si>
+    <t>Galvanized Steel</t>
   </si>
 </sst>
 </file>
@@ -477,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CDE8C3E-D2CD-4FEC-B8FA-734CEE576120}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" bestFit="1" customWidth="1"/>
@@ -807,6 +810,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20">
+        <v>30000000</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0</v>
+      </c>
+      <c r="D20" s="1">
+        <v>40000</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed Spring PRBM and Added a spreadsheet for forces and safety factors for certain geometries
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D76C94-FCC6-4518-AE59-C19DA35C5E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1716E47A-4F94-4D9E-8ED3-CC08DA4685E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Material</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>Galvanized Steel</t>
+  </si>
+  <si>
+    <t>Polycarbonate</t>
   </si>
 </sst>
 </file>
@@ -480,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CDE8C3E-D2CD-4FEC-B8FA-734CEE576120}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" bestFit="1" customWidth="1"/>
@@ -659,84 +662,84 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11">
-        <v>400000</v>
+        <v>200000</v>
       </c>
       <c r="C11" s="1">
-        <v>2800000000</v>
+        <v>1400000000</v>
       </c>
       <c r="D11" s="1">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="E11" s="1">
-        <v>55000000</v>
+        <v>34000000</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B12">
-        <v>200000</v>
+        <v>12000000</v>
       </c>
       <c r="C12" s="1">
-        <v>1400000000</v>
+        <v>86000000000</v>
       </c>
       <c r="D12" s="1">
-        <v>5000</v>
+        <v>220000</v>
       </c>
       <c r="E12" s="1">
-        <v>34000000</v>
+        <v>1517000000</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B13">
-        <v>12000000</v>
+        <v>8100000</v>
       </c>
       <c r="C13" s="1">
-        <v>86000000000</v>
+        <v>56000000000</v>
       </c>
       <c r="D13" s="1">
-        <v>220000</v>
+        <v>238000</v>
       </c>
       <c r="E13" s="1">
-        <v>1517000000</v>
+        <v>1640000000</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B14">
-        <v>8100000</v>
+        <v>400000</v>
       </c>
       <c r="C14" s="1">
-        <v>56000000000</v>
+        <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>238000</v>
+        <v>8000</v>
       </c>
       <c r="E14" s="1">
-        <v>1640000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15">
-        <v>400000</v>
+        <v>20</v>
+      </c>
+      <c r="B15" s="1">
+        <v>325000</v>
       </c>
       <c r="C15" s="1">
         <v>0</v>
       </c>
       <c r="D15" s="1">
-        <v>8000</v>
+        <v>7000</v>
       </c>
       <c r="E15" s="1">
         <v>0</v>
@@ -744,16 +747,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16">
-        <v>500000</v>
+        <v>21</v>
+      </c>
+      <c r="B16" s="1">
+        <v>28000000</v>
       </c>
       <c r="C16" s="1">
-        <v>3250000000</v>
+        <v>0</v>
       </c>
       <c r="D16" s="1">
-        <v>12000</v>
+        <v>45000</v>
       </c>
       <c r="E16" s="1">
         <v>0</v>
@@ -761,16 +764,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B17" s="1">
-        <v>325000</v>
+        <v>28000000</v>
       </c>
       <c r="C17" s="1">
         <v>0</v>
       </c>
       <c r="D17" s="1">
-        <v>7000</v>
+        <v>29700</v>
       </c>
       <c r="E17" s="1">
         <v>0</v>
@@ -778,16 +781,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="1">
-        <v>28000000</v>
+        <v>23</v>
+      </c>
+      <c r="B18">
+        <v>30000000</v>
       </c>
       <c r="C18" s="1">
         <v>0</v>
       </c>
       <c r="D18" s="1">
-        <v>45000</v>
+        <v>40000</v>
       </c>
       <c r="E18" s="1">
         <v>0</v>
@@ -795,36 +798,56 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B19" s="1">
-        <v>28000000</v>
+        <v>325000</v>
       </c>
       <c r="C19" s="1">
-        <v>0</v>
+        <f>B19*6895</f>
+        <v>2240875000</v>
       </c>
       <c r="D19" s="1">
-        <v>29700</v>
+        <f>E19/6895</f>
+        <v>14068.16533720087</v>
       </c>
       <c r="E19" s="1">
-        <v>0</v>
+        <v>97000000</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B20">
-        <v>30000000</v>
+        <v>500000</v>
       </c>
       <c r="C20" s="1">
-        <v>0</v>
+        <v>3250000000</v>
       </c>
       <c r="D20" s="1">
-        <v>40000</v>
+        <v>12000</v>
       </c>
       <c r="E20" s="1">
-        <v>0</v>
+        <f>D20*6895</f>
+        <v>82740000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21">
+        <v>400000</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2800000000</v>
+      </c>
+      <c r="D21" s="1">
+        <v>8000</v>
+      </c>
+      <c r="E21" s="1">
+        <v>55000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Documented lots of the previous scripts and created some scripts for organization of final design package.
</commit_message>
<xml_diff>
--- a/Capstone/BookMaterials.xlsx
+++ b/Capstone/BookMaterials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\Capstone\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1716E47A-4F94-4D9E-8ED3-CC08DA4685E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF22867B-9313-4372-9171-F649A5B0B942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1716AEB-2E5E-43B7-950F-41B1B686F8EF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Material</t>
   </si>
@@ -77,13 +77,7 @@
     <t>E (psi)</t>
   </si>
   <si>
-    <t>E (Pa)</t>
-  </si>
-  <si>
     <t>Sy (psi)</t>
-  </si>
-  <si>
-    <t>Sy (Pa)</t>
   </si>
   <si>
     <t>Kevlar (82 vol % in epoxy)</t>
@@ -500,12 +494,6 @@
       <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" t="s">
-        <v>15</v>
-      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -514,32 +502,22 @@
       <c r="B2">
         <v>30000000</v>
       </c>
-      <c r="C2">
-        <v>207000000000</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="C2" s="1">
         <v>26000</v>
       </c>
-      <c r="E2" s="1">
-        <v>179000000</v>
-      </c>
+      <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B3">
         <v>30000000</v>
       </c>
       <c r="C3" s="1">
-        <v>207000000000</v>
-      </c>
-      <c r="D3" s="1">
         <v>238000</v>
       </c>
-      <c r="E3" s="1">
-        <v>1641000000</v>
-      </c>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -549,14 +527,9 @@
         <v>10400000</v>
       </c>
       <c r="C4" s="1">
-        <v>71700000000</v>
-      </c>
-      <c r="D4" s="1">
         <v>5000</v>
       </c>
-      <c r="E4" s="1">
-        <v>34000000</v>
-      </c>
+      <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -566,14 +539,9 @@
         <v>10400000</v>
       </c>
       <c r="C5" s="1">
-        <v>71700000000</v>
-      </c>
-      <c r="D5" s="1">
         <v>73000</v>
       </c>
-      <c r="E5" s="1">
-        <v>503000000</v>
-      </c>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -583,14 +551,9 @@
         <v>16500000</v>
       </c>
       <c r="C6" s="1">
-        <v>114000000000</v>
-      </c>
-      <c r="D6" s="1">
         <v>30000</v>
       </c>
-      <c r="E6" s="1">
-        <v>207000000</v>
-      </c>
+      <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -600,14 +563,9 @@
         <v>16500000</v>
       </c>
       <c r="C7" s="1">
-        <v>114000000000</v>
-      </c>
-      <c r="D7" s="1">
         <v>170000</v>
       </c>
-      <c r="E7" s="1">
-        <v>1170000000</v>
-      </c>
+      <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -617,14 +575,9 @@
         <v>18500000</v>
       </c>
       <c r="C8" s="1">
-        <v>128000000000</v>
-      </c>
-      <c r="D8" s="1">
         <v>170000</v>
       </c>
-      <c r="E8" s="1">
-        <v>1170000000</v>
-      </c>
+      <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -634,14 +587,9 @@
         <v>24500000</v>
       </c>
       <c r="C9" s="1">
-        <v>169000000000</v>
-      </c>
-      <c r="D9" s="1">
         <v>135000</v>
       </c>
-      <c r="E9" s="1">
-        <v>930000000</v>
-      </c>
+      <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -651,14 +599,9 @@
         <v>200000</v>
       </c>
       <c r="C10" s="1">
-        <v>1400000000</v>
-      </c>
-      <c r="D10" s="1">
         <v>4000</v>
       </c>
-      <c r="E10" s="1">
-        <v>28000000</v>
-      </c>
+      <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -668,31 +611,21 @@
         <v>200000</v>
       </c>
       <c r="C11" s="1">
-        <v>1400000000</v>
-      </c>
-      <c r="D11" s="1">
         <v>5000</v>
       </c>
-      <c r="E11" s="1">
-        <v>34000000</v>
-      </c>
+      <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>12000000</v>
       </c>
       <c r="C12" s="1">
-        <v>86000000000</v>
-      </c>
-      <c r="D12" s="1">
         <v>220000</v>
       </c>
-      <c r="E12" s="1">
-        <v>1517000000</v>
-      </c>
+      <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -702,136 +635,94 @@
         <v>8100000</v>
       </c>
       <c r="C13" s="1">
-        <v>56000000000</v>
-      </c>
-      <c r="D13" s="1">
         <v>238000</v>
       </c>
-      <c r="E13" s="1">
-        <v>1640000000</v>
-      </c>
+      <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>400000</v>
       </c>
       <c r="C14" s="1">
-        <v>0</v>
-      </c>
-      <c r="D14" s="1">
         <v>8000</v>
       </c>
-      <c r="E14" s="1">
-        <v>0</v>
-      </c>
+      <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B15" s="1">
         <v>325000</v>
       </c>
       <c r="C15" s="1">
-        <v>0</v>
-      </c>
-      <c r="D15" s="1">
         <v>7000</v>
       </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
+      <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1">
         <v>28000000</v>
       </c>
       <c r="C16" s="1">
-        <v>0</v>
-      </c>
-      <c r="D16" s="1">
         <v>45000</v>
       </c>
-      <c r="E16" s="1">
-        <v>0</v>
-      </c>
+      <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1">
         <v>28000000</v>
       </c>
       <c r="C17" s="1">
-        <v>0</v>
-      </c>
-      <c r="D17" s="1">
         <v>29700</v>
       </c>
-      <c r="E17" s="1">
-        <v>0</v>
-      </c>
+      <c r="E17" s="1"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B18">
         <v>30000000</v>
       </c>
       <c r="C18" s="1">
-        <v>0</v>
-      </c>
-      <c r="D18" s="1">
         <v>40000</v>
       </c>
-      <c r="E18" s="1">
-        <v>0</v>
-      </c>
+      <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B19" s="1">
         <v>325000</v>
       </c>
       <c r="C19" s="1">
-        <f>B19*6895</f>
-        <v>2240875000</v>
-      </c>
-      <c r="D19" s="1">
         <f>E19/6895</f>
-        <v>14068.16533720087</v>
-      </c>
-      <c r="E19" s="1">
-        <v>97000000</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B20">
         <v>500000</v>
       </c>
       <c r="C20" s="1">
-        <v>3250000000</v>
-      </c>
-      <c r="D20" s="1">
         <v>12000</v>
       </c>
-      <c r="E20" s="1">
-        <f>D20*6895</f>
-        <v>82740000</v>
-      </c>
+      <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
@@ -841,14 +732,9 @@
         <v>400000</v>
       </c>
       <c r="C21" s="1">
-        <v>2800000000</v>
-      </c>
-      <c r="D21" s="1">
         <v>8000</v>
       </c>
-      <c r="E21" s="1">
-        <v>55000000</v>
-      </c>
+      <c r="E21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>